<commit_message>
vault backup: 2026-02-20 11:25:54
</commit_message>
<xml_diff>
--- a/FY1/1/FY1 - LAB1.xlsx
+++ b/FY1/1/FY1 - LAB1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marian/Documents/Zapisky/FY1/1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41573ED4-A0BE-414A-AD1F-9B5DFD7049B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDBD0F0-3F60-804F-BC18-F5CF1440DF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{50D1F2D1-F177-9540-9CCC-CA14B3043CC0}"/>
   </bookViews>
@@ -35,15 +35,148 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="41">
+  <si>
+    <t>Marian Frýba</t>
+  </si>
+  <si>
+    <t>Válec</t>
+  </si>
+  <si>
+    <t>Hranol</t>
+  </si>
+  <si>
+    <t>Měření:</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>11,78mm</t>
+  </si>
+  <si>
+    <t>11,66mm</t>
+  </si>
+  <si>
+    <t>11,6mm</t>
+  </si>
+  <si>
+    <t>11,7mm</t>
+  </si>
+  <si>
+    <t>11,68mm</t>
+  </si>
+  <si>
+    <t>11,64mm</t>
+  </si>
+  <si>
+    <t>27,5mm</t>
+  </si>
+  <si>
+    <t>27,46mm</t>
+  </si>
+  <si>
+    <t>27,52mm</t>
+  </si>
+  <si>
+    <t>27,48mm</t>
+  </si>
+  <si>
+    <t>27,44mm</t>
+  </si>
+  <si>
+    <t>31,54mm</t>
+  </si>
+  <si>
+    <t>31,52mm</t>
+  </si>
+  <si>
+    <t>31,5mm</t>
+  </si>
+  <si>
+    <t>31,56mm</t>
+  </si>
+  <si>
+    <t>Arit. Průměr</t>
+  </si>
+  <si>
+    <t>Arit. průměr:</t>
+  </si>
+  <si>
+    <t>31,68mm</t>
+  </si>
+  <si>
+    <t>31,62mm</t>
+  </si>
+  <si>
+    <t>31,7mm</t>
+  </si>
+  <si>
+    <t>13,72mm</t>
+  </si>
+  <si>
+    <t>13,6mm</t>
+  </si>
+  <si>
+    <t>13,64mm</t>
+  </si>
+  <si>
+    <t>13,68mm</t>
+  </si>
+  <si>
+    <t>13,66mm</t>
+  </si>
+  <si>
+    <t>13,62mm</t>
+  </si>
+  <si>
+    <t>13,7mm</t>
+  </si>
+  <si>
+    <t>13,76mm</t>
+  </si>
+  <si>
+    <t>20mm</t>
+  </si>
+  <si>
+    <t>20,02mm</t>
+  </si>
+  <si>
+    <t>19,98mm</t>
+  </si>
+  <si>
+    <t>20,06mm</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
   <fills count="2">
@@ -54,7 +187,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -62,12 +195,261 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,9 +784,306 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{468333C8-8064-D14E-96D6-F476956B8A12}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:8" ht="32" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="1"/>
+    </row>
+    <row r="2" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="18"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="17" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="19"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A3" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="13">
+        <v>1</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="13">
+        <v>1</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G4" s="14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" s="13">
+        <v>2</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="13">
+        <v>2</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="13">
+        <v>3</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" s="13">
+        <v>3</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" s="13">
+        <v>4</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="13">
+        <v>4</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="13">
+        <v>5</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="13">
+        <v>5</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="14" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" s="13">
+        <v>6</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" s="13">
+        <v>6</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="13">
+        <v>7</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="13">
+        <v>7</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" s="13">
+        <v>8</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="13">
+        <v>8</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="G11" s="14" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="13">
+        <v>9</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="D12" s="13">
+        <v>9</v>
+      </c>
+      <c r="E12" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="G12" s="14" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="15">
+        <v>10</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="15">
+        <v>10</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="16" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
vault backup: 2026-03-06 10:41:16
</commit_message>
<xml_diff>
--- a/FY1/1/FY1 - LAB1.xlsx
+++ b/FY1/1/FY1 - LAB1.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marian/Documents/Zapisky/FY1/1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CDBD0F0-3F60-804F-BC18-F5CF1440DF5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18316CE2-6281-F145-A998-32A29021E89F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{50D1F2D1-F177-9540-9CCC-CA14B3043CC0}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{50D1F2D1-F177-9540-9CCC-CA14B3043CC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>Marian Frýba</t>
   </si>
@@ -50,115 +50,25 @@
     <t>Měření:</t>
   </si>
   <si>
-    <t>d</t>
-  </si>
-  <si>
-    <t>h</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>b</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>11,78mm</t>
-  </si>
-  <si>
-    <t>11,66mm</t>
-  </si>
-  <si>
-    <t>11,6mm</t>
-  </si>
-  <si>
-    <t>11,7mm</t>
-  </si>
-  <si>
-    <t>11,68mm</t>
-  </si>
-  <si>
-    <t>11,64mm</t>
-  </si>
-  <si>
-    <t>27,5mm</t>
-  </si>
-  <si>
-    <t>27,46mm</t>
-  </si>
-  <si>
-    <t>27,52mm</t>
-  </si>
-  <si>
-    <t>27,48mm</t>
-  </si>
-  <si>
-    <t>27,44mm</t>
-  </si>
-  <si>
-    <t>31,54mm</t>
-  </si>
-  <si>
-    <t>31,52mm</t>
-  </si>
-  <si>
-    <t>31,5mm</t>
-  </si>
-  <si>
-    <t>31,56mm</t>
-  </si>
-  <si>
     <t>Arit. Průměr</t>
   </si>
   <si>
     <t>Arit. průměr:</t>
   </si>
   <si>
-    <t>31,68mm</t>
+    <t>d(mm)</t>
   </si>
   <si>
-    <t>31,62mm</t>
+    <t>h(mm)</t>
   </si>
   <si>
-    <t>31,7mm</t>
+    <t>a(mm)</t>
   </si>
   <si>
-    <t>13,72mm</t>
+    <t>b(mm)</t>
   </si>
   <si>
-    <t>13,6mm</t>
-  </si>
-  <si>
-    <t>13,64mm</t>
-  </si>
-  <si>
-    <t>13,68mm</t>
-  </si>
-  <si>
-    <t>13,66mm</t>
-  </si>
-  <si>
-    <t>13,62mm</t>
-  </si>
-  <si>
-    <t>13,7mm</t>
-  </si>
-  <si>
-    <t>13,76mm</t>
-  </si>
-  <si>
-    <t>20mm</t>
-  </si>
-  <si>
-    <t>20,02mm</t>
-  </si>
-  <si>
-    <t>19,98mm</t>
-  </si>
-  <si>
-    <t>20,06mm</t>
+    <t>c(mm)</t>
   </si>
 </sst>
 </file>
@@ -417,16 +327,7 @@
   </cellStyleXfs>
   <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
@@ -448,6 +349,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -788,295 +698,310 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="4"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="19"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="18"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="17" t="s">
+      <c r="B2" s="15"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="19"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="16"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="10">
+        <v>1</v>
+      </c>
+      <c r="B4" s="6">
+        <v>13.72</v>
+      </c>
+      <c r="C4" s="11">
+        <v>20</v>
+      </c>
+      <c r="D4" s="10">
+        <v>1</v>
+      </c>
+      <c r="E4" s="6">
+        <v>11.78</v>
+      </c>
+      <c r="F4" s="6">
+        <v>27.5</v>
+      </c>
+      <c r="G4" s="11">
+        <v>31.54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A5" s="10">
+        <v>2</v>
+      </c>
+      <c r="B5" s="6">
+        <v>13.6</v>
+      </c>
+      <c r="C5" s="11">
+        <v>20.02</v>
+      </c>
+      <c r="D5" s="10">
+        <v>2</v>
+      </c>
+      <c r="E5" s="6">
+        <v>11.66</v>
+      </c>
+      <c r="F5" s="6">
+        <v>27.46</v>
+      </c>
+      <c r="G5" s="11">
+        <v>31.52</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A6" s="10">
+        <v>3</v>
+      </c>
+      <c r="B6" s="6">
+        <v>13.64</v>
+      </c>
+      <c r="C6" s="11">
+        <v>20</v>
+      </c>
+      <c r="D6" s="10">
+        <v>3</v>
+      </c>
+      <c r="E6" s="6">
+        <v>11.78</v>
+      </c>
+      <c r="F6" s="6">
+        <v>27.52</v>
+      </c>
+      <c r="G6" s="11">
+        <v>31.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A7" s="10">
         <v>4</v>
       </c>
-      <c r="C3" s="12" t="s">
+      <c r="B7" s="6">
+        <v>13.68</v>
+      </c>
+      <c r="C7" s="11">
+        <v>19.98</v>
+      </c>
+      <c r="D7" s="10">
+        <v>4</v>
+      </c>
+      <c r="E7" s="6">
+        <v>11.6</v>
+      </c>
+      <c r="F7" s="6">
+        <v>27.5</v>
+      </c>
+      <c r="G7" s="11">
+        <v>31.52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A8" s="10">
         <v>5</v>
       </c>
-      <c r="D3" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="E3" s="8" t="s">
+      <c r="B8" s="6">
+        <v>13.66</v>
+      </c>
+      <c r="C8" s="11">
+        <v>20.059999999999999</v>
+      </c>
+      <c r="D8" s="10">
+        <v>5</v>
+      </c>
+      <c r="E8" s="6">
+        <v>11.7</v>
+      </c>
+      <c r="F8" s="6">
+        <v>27.48</v>
+      </c>
+      <c r="G8" s="11">
+        <v>31.56</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A9" s="10">
         <v>6</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="B9" s="6">
+        <v>13.62</v>
+      </c>
+      <c r="C9" s="11">
+        <v>20.02</v>
+      </c>
+      <c r="D9" s="10">
+        <v>6</v>
+      </c>
+      <c r="E9" s="6">
+        <v>11.68</v>
+      </c>
+      <c r="F9" s="6">
+        <v>27.44</v>
+      </c>
+      <c r="G9" s="11">
+        <v>31.54</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A10" s="10">
         <v>7</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="B10" s="6">
+        <v>13.62</v>
+      </c>
+      <c r="C10" s="11">
+        <v>20</v>
+      </c>
+      <c r="D10" s="10">
+        <v>7</v>
+      </c>
+      <c r="E10" s="6">
+        <v>11.64</v>
+      </c>
+      <c r="F10" s="6">
+        <v>27.46</v>
+      </c>
+      <c r="G10" s="11">
+        <v>31.68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A11" s="10">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="13">
-        <v>1</v>
-      </c>
-      <c r="B4" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D4" s="13">
-        <v>1</v>
-      </c>
-      <c r="E4" s="9" t="s">
+      <c r="B11" s="6">
+        <v>13.7</v>
+      </c>
+      <c r="C11" s="11">
+        <v>20.02</v>
+      </c>
+      <c r="D11" s="10">
+        <v>8</v>
+      </c>
+      <c r="E11" s="6">
+        <v>11.7</v>
+      </c>
+      <c r="F11" s="6">
+        <v>27.48</v>
+      </c>
+      <c r="G11" s="11">
+        <v>31.52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A12" s="10">
         <v>9</v>
       </c>
-      <c r="F4" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="14" t="s">
+      <c r="B12" s="6">
+        <v>13.76</v>
+      </c>
+      <c r="C12" s="11">
         <v>20</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A5" s="13">
-        <v>2</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="C5" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D5" s="13">
-        <v>2</v>
-      </c>
-      <c r="E5" s="9" t="s">
+      <c r="D12" s="10">
+        <v>9</v>
+      </c>
+      <c r="E12" s="6">
+        <v>11.68</v>
+      </c>
+      <c r="F12" s="6">
+        <v>27.5</v>
+      </c>
+      <c r="G12" s="11">
+        <v>31.62</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A13" s="12">
         <v>10</v>
       </c>
-      <c r="F5" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" s="13">
-        <v>3</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D6" s="13">
-        <v>3</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="G6" s="14" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A7" s="13">
+      <c r="B13" s="7">
+        <v>13.72</v>
+      </c>
+      <c r="C13" s="13">
+        <v>19.98</v>
+      </c>
+      <c r="D13" s="12">
+        <v>10</v>
+      </c>
+      <c r="E13" s="7">
+        <v>11.78</v>
+      </c>
+      <c r="F13" s="7">
+        <v>27.52</v>
+      </c>
+      <c r="G13" s="13">
+        <v>31.7</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="13">
-        <v>4</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F7" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A8" s="13">
+      <c r="B14" s="3">
+        <f>AVERAGE(B4:B13)</f>
+        <v>13.672000000000002</v>
+      </c>
+      <c r="C14" s="4">
+        <f>AVERAGE(C4:C13)</f>
+        <v>20.007999999999999</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="13">
-        <v>5</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A9" s="13">
-        <v>6</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="13">
-        <v>6</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A10" s="13">
-        <v>7</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D10" s="13">
-        <v>7</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="F10" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A11" s="13">
-        <v>8</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="13">
-        <v>8</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="G11" s="14" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A12" s="13">
-        <v>9</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="13">
-        <v>9</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F12" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A13" s="15">
-        <v>10</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C13" s="16" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="15">
-        <v>10</v>
-      </c>
-      <c r="E13" s="10" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="G13" s="16" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="7"/>
+      <c r="E14" s="3">
+        <f>AVERAGE(E4:E13)</f>
+        <v>11.7</v>
+      </c>
+      <c r="F14" s="3">
+        <f>AVERAGE(F4:F13)</f>
+        <v>27.486000000000001</v>
+      </c>
+      <c r="G14" s="4">
+        <f>AVERAGE(G4:G13)</f>
+        <v>31.57</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
vault backup: 2026-03-07 22:47:29
</commit_message>
<xml_diff>
--- a/FY1/1/FY1 - LAB1.xlsx
+++ b/FY1/1/FY1 - LAB1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marian/Documents/Zapisky/FY1/1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D1A97E8-860C-DD41-9CA1-CC79E050000A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A93E30F-EFA9-2448-AA0F-D59F4FDB6EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{50D1F2D1-F177-9540-9CCC-CA14B3043CC0}"/>
   </bookViews>
@@ -71,16 +71,16 @@
     <t>Arit. Průměr:</t>
   </si>
   <si>
-    <t>Nejpravděpodb. objem(mm³):</t>
-  </si>
-  <si>
     <t>Nejistota typu A:</t>
   </si>
   <si>
     <t>Kombinovaná nejistota:</t>
   </si>
   <si>
-    <t>Nejistota typu B (měření probíhalo pouze posuvným měřítkem (odchylka 20μm):</t>
+    <t xml:space="preserve">                                                                           Nejistota typu B (měření probíhalo v obou případech posuvným měřítkem (odchylka 20μm):</t>
+  </si>
+  <si>
+    <t>Nejpravděpodbnější objem(mm³):</t>
   </si>
 </sst>
 </file>
@@ -109,7 +109,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -164,17 +164,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
@@ -352,9 +341,7 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -478,16 +465,58 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
@@ -495,14 +524,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -514,14 +542,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -531,15 +557,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -547,53 +576,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -601,8 +585,59 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -736,9 +771,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>883186</xdr:colOff>
+      <xdr:colOff>1117133</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>100830</xdr:rowOff>
+      <xdr:rowOff>111971</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="770659" cy="181460"/>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -756,7 +791,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8001870" y="4389865"/>
+              <a:off x="8235817" y="4401006"/>
               <a:ext cx="770659" cy="181460"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -920,7 +955,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="8001870" y="4389865"/>
+              <a:off x="8235817" y="4401006"/>
               <a:ext cx="770659" cy="181460"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -972,9 +1007,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>658860</xdr:colOff>
+      <xdr:colOff>903948</xdr:colOff>
       <xdr:row>16</xdr:row>
-      <xdr:rowOff>43103</xdr:rowOff>
+      <xdr:rowOff>20822</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="897362" cy="316882"/>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -992,7 +1027,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="1928860" y="3179618"/>
+              <a:off x="2296492" y="4309857"/>
               <a:ext cx="897362" cy="316882"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -1181,7 +1216,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="1928860" y="3179618"/>
+              <a:off x="2296492" y="4309857"/>
               <a:ext cx="897362" cy="316882"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -1245,10 +1280,10 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>93489</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1073840</xdr:colOff>
       <xdr:row>17</xdr:row>
-      <xdr:rowOff>41584</xdr:rowOff>
+      <xdr:rowOff>30444</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="1986378" cy="523348"/>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -1266,7 +1301,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="9507085" y="4720531"/>
+              <a:off x="8192524" y="4709391"/>
               <a:ext cx="1986378" cy="523348"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -1516,7 +1551,7 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="9507085" y="4720531"/>
+              <a:off x="8192524" y="4709391"/>
               <a:ext cx="1986378" cy="523348"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
@@ -2736,12 +2771,12 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>490681</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>212172</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>139314</xdr:rowOff>
+      <xdr:rowOff>50191</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5042471" cy="500137"/>
+    <xdr:ext cx="4270592" cy="677301"/>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
@@ -2757,8 +2792,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="490681" y="6065981"/>
-              <a:ext cx="5042471" cy="500137"/>
+              <a:off x="1604716" y="5943437"/>
+              <a:ext cx="4270592" cy="677301"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3113,6 +3148,20 @@
                         </m:sSup>
                       </m:e>
                     </m:rad>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                     <m:r>
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -3178,8 +3227,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="490681" y="6065981"/>
-              <a:ext cx="5042471" cy="500137"/>
+              <a:off x="1604716" y="5943437"/>
+              <a:ext cx="4270592" cy="677301"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3210,7 +3259,18 @@
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>𝑢_𝐶 (¯𝑉)=√((𝜋^2⋅〖13,672〗^4)/16⋅〖0,00940〗^2+(𝜋^2⋅〖13,672〗^2⋅〖20,008〗^2)/4⋅〖0,01763〗^2 )≈7,70" " 〖"mm" 〗^3</a:t>
+                <a:t>𝑢_𝐶 (¯𝑉)=√((𝜋^2⋅〖13,672〗^4)/16⋅〖0,00940〗^2+(𝜋^2⋅〖13,672〗^2⋅〖20,008〗^2)/4⋅〖0,01763〗^2 )</a:t>
+              </a:r>
+              <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>≈7,70" " 〖"mm" 〗^3</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -3222,12 +3282,12 @@
   </xdr:oneCellAnchor>
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>356806</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>278824</xdr:colOff>
       <xdr:row>19</xdr:row>
-      <xdr:rowOff>244644</xdr:rowOff>
+      <xdr:rowOff>166662</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="7246920" cy="215252"/>
+    <xdr:ext cx="6396944" cy="392415"/>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
@@ -3243,8 +3303,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6383736" y="6137890"/>
-              <a:ext cx="7246920" cy="215252"/>
+              <a:off x="7397508" y="6059908"/>
+              <a:ext cx="6396944" cy="392415"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3563,6 +3623,20 @@
                         </m:sSup>
                       </m:e>
                     </m:rad>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                     <m:r>
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -3628,8 +3702,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="6383736" y="6137890"/>
-              <a:ext cx="7246920" cy="215252"/>
+              <a:off x="7397508" y="6059908"/>
+              <a:ext cx="6396944" cy="392415"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3660,7 +3734,18 @@
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>𝑢_𝐶 (¯𝑉)=√((27,486⋅31,570)^2⋅〖0,02060〗^2+(11,700⋅31,570)^2⋅〖0,01024〗^2+(11,700⋅27,486)^2⋅〖0,02329〗^2 )≈19,75" " 〖"mm" 〗^3</a:t>
+                <a:t>𝑢_𝐶 (¯𝑉)=√((27,486⋅31,570)^2⋅〖0,02060〗^2+(11,700⋅31,570)^2⋅〖0,01024〗^2+(11,700⋅27,486)^2⋅〖0,02329〗^2 )</a:t>
+              </a:r>
+              <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>≈19,75" " 〖"mm" 〗^3</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -6087,25 +6172,25 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="21">
+      <c r="A4" s="19">
         <v>1</v>
       </c>
-      <c r="B4" s="18">
+      <c r="B4" s="17">
         <v>13.72</v>
       </c>
-      <c r="C4" s="22">
+      <c r="C4" s="20">
         <v>20</v>
       </c>
-      <c r="D4" s="21">
+      <c r="D4" s="19">
         <v>1</v>
       </c>
-      <c r="E4" s="18">
+      <c r="E4" s="17">
         <v>11.78</v>
       </c>
-      <c r="F4" s="23">
+      <c r="F4" s="21">
         <v>27.5</v>
       </c>
-      <c r="G4" s="22">
+      <c r="G4" s="20">
         <v>31.54</v>
       </c>
     </row>
@@ -6125,7 +6210,7 @@
       <c r="E5" s="3">
         <v>11.66</v>
       </c>
-      <c r="F5" s="24">
+      <c r="F5" s="22">
         <v>27.46</v>
       </c>
       <c r="G5" s="8">
@@ -6148,7 +6233,7 @@
       <c r="E6" s="3">
         <v>11.78</v>
       </c>
-      <c r="F6" s="24">
+      <c r="F6" s="22">
         <v>27.52</v>
       </c>
       <c r="G6" s="8">
@@ -6171,7 +6256,7 @@
       <c r="E7" s="3">
         <v>11.6</v>
       </c>
-      <c r="F7" s="24">
+      <c r="F7" s="22">
         <v>27.5</v>
       </c>
       <c r="G7" s="8">
@@ -6194,7 +6279,7 @@
       <c r="E8" s="3">
         <v>11.7</v>
       </c>
-      <c r="F8" s="24">
+      <c r="F8" s="22">
         <v>27.48</v>
       </c>
       <c r="G8" s="8">
@@ -6217,7 +6302,7 @@
       <c r="E9" s="3">
         <v>11.68</v>
       </c>
-      <c r="F9" s="24">
+      <c r="F9" s="22">
         <v>27.44</v>
       </c>
       <c r="G9" s="8">
@@ -6240,7 +6325,7 @@
       <c r="E10" s="3">
         <v>11.64</v>
       </c>
-      <c r="F10" s="24">
+      <c r="F10" s="22">
         <v>27.46</v>
       </c>
       <c r="G10" s="8">
@@ -6263,7 +6348,7 @@
       <c r="E11" s="3">
         <v>11.7</v>
       </c>
-      <c r="F11" s="24">
+      <c r="F11" s="22">
         <v>27.48</v>
       </c>
       <c r="G11" s="8">
@@ -6286,7 +6371,7 @@
       <c r="E12" s="3">
         <v>11.68</v>
       </c>
-      <c r="F12" s="24">
+      <c r="F12" s="22">
         <v>27.5</v>
       </c>
       <c r="G12" s="8">
@@ -6309,7 +6394,7 @@
       <c r="E13" s="4">
         <v>11.78</v>
       </c>
-      <c r="F13" s="20">
+      <c r="F13" s="18">
         <v>27.52</v>
       </c>
       <c r="G13" s="10">
@@ -6335,7 +6420,7 @@
         <f>AVERAGE(E4:E13)</f>
         <v>11.7</v>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="18">
         <f>AVERAGE(F4:F13)</f>
         <v>27.486000000000001</v>
       </c>
@@ -6345,140 +6430,140 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="35" t="s">
-        <v>12</v>
-      </c>
-      <c r="B15" s="43"/>
-      <c r="C15" s="45"/>
-      <c r="D15" s="41" t="s">
-        <v>12</v>
-      </c>
-      <c r="E15" s="47"/>
-      <c r="F15" s="43"/>
-      <c r="G15" s="38"/>
+      <c r="A15" s="34" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="39"/>
+      <c r="C15" s="40"/>
+      <c r="D15" s="38" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="41"/>
+      <c r="F15" s="39"/>
+      <c r="G15" s="37"/>
     </row>
-    <row r="16" spans="1:8" ht="39" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="36"/>
-      <c r="B16" s="44"/>
-      <c r="C16" s="46"/>
-      <c r="D16" s="42"/>
-      <c r="E16" s="48"/>
-      <c r="F16" s="44"/>
-      <c r="G16" s="31"/>
+    <row r="16" spans="1:8" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="35"/>
+      <c r="B16" s="48"/>
+      <c r="C16" s="49"/>
+      <c r="D16" s="50"/>
+      <c r="E16" s="51"/>
+      <c r="F16" s="48"/>
+      <c r="G16" s="26"/>
     </row>
     <row r="17" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="34">
+      <c r="A17" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="29"/>
+      <c r="C17" s="52">
         <f>0.25*PI()*POWER(B14,2)*C14</f>
         <v>2937.363266901928</v>
       </c>
-      <c r="D17" s="32" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" s="33"/>
-      <c r="F17" s="33"/>
-      <c r="G17" s="34">
+      <c r="D17" s="28" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="53"/>
+      <c r="F17" s="12">
         <f>E14*F14*G14</f>
         <v>10152.476333999999</v>
       </c>
+      <c r="G17" s="13"/>
     </row>
     <row r="18" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="39" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" s="40"/>
-      <c r="C18" s="40"/>
-      <c r="D18" s="50"/>
-      <c r="E18" s="50"/>
-      <c r="F18" s="50"/>
-      <c r="G18" s="51"/>
+      <c r="A18" s="30" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="31"/>
+      <c r="C18" s="31"/>
+      <c r="D18" s="32"/>
+      <c r="E18" s="32"/>
+      <c r="F18" s="32"/>
+      <c r="G18" s="33"/>
     </row>
     <row r="19" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="49" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="52" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="38"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
+      <c r="A19" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="B19" s="42"/>
+      <c r="C19" s="44"/>
+      <c r="D19" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="27"/>
+      <c r="I19" s="27"/>
+      <c r="J19" s="27"/>
     </row>
     <row r="20" spans="1:10" ht="61" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="17"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="27"/>
-      <c r="F20" s="27"/>
-      <c r="G20" s="28"/>
-      <c r="H20" s="25"/>
-      <c r="I20" s="25"/>
+      <c r="A20" s="47"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="45"/>
+      <c r="D20" s="47"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="24"/>
+      <c r="G20" s="25"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" s="30"/>
-      <c r="B21" s="30"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30"/>
-      <c r="E21" s="30"/>
-      <c r="F21" s="30"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-      <c r="I21" s="30"/>
+      <c r="A21" s="27"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="27"/>
+      <c r="D21" s="27"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="27"/>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="30"/>
-      <c r="B22" s="30"/>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30"/>
-      <c r="E22" s="30"/>
-      <c r="F22" s="30"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-      <c r="I22" s="30"/>
+      <c r="A22" s="27"/>
+      <c r="B22" s="27"/>
+      <c r="C22" s="27"/>
+      <c r="D22" s="27"/>
+      <c r="E22" s="27"/>
+      <c r="F22" s="27"/>
+      <c r="G22" s="27"/>
+      <c r="H22" s="27"/>
+      <c r="I22" s="27"/>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="30"/>
-      <c r="B23" s="30"/>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="30"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="30"/>
+      <c r="A23" s="27"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="27"/>
+      <c r="G23" s="27"/>
+      <c r="H23" s="27"/>
+      <c r="I23" s="27"/>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="30"/>
-      <c r="B24" s="30"/>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="30"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="30"/>
+      <c r="A24" s="27"/>
+      <c r="B24" s="27"/>
+      <c r="C24" s="27"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="27"/>
+      <c r="G24" s="27"/>
+      <c r="H24" s="27"/>
+      <c r="I24" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="17">
+  <mergeCells count="18">
+    <mergeCell ref="D17:E17"/>
     <mergeCell ref="A18:G18"/>
-    <mergeCell ref="B19:C19"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="E19:G19"/>
-    <mergeCell ref="D20:G20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:C20"/>
+    <mergeCell ref="E19:G20"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="D2:G2"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A17:B17"/>
-    <mergeCell ref="D17:F17"/>
     <mergeCell ref="D15:D16"/>
     <mergeCell ref="A15:A16"/>
     <mergeCell ref="B15:B16"/>
@@ -6486,6 +6571,7 @@
     <mergeCell ref="G15:G16"/>
     <mergeCell ref="F15:F16"/>
     <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F17:G17"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-13 13:36:54
</commit_message>
<xml_diff>
--- a/FY1/1/FY1 - LAB1.xlsx
+++ b/FY1/1/FY1 - LAB1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marian/Documents/Zapisky/FY1/1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A93E30F-EFA9-2448-AA0F-D59F4FDB6EAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74CEBC7E-243B-1145-ABAC-24D070CB8BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{50D1F2D1-F177-9540-9CCC-CA14B3043CC0}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{50D1F2D1-F177-9540-9CCC-CA14B3043CC0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -74,13 +74,13 @@
     <t>Nejistota typu A:</t>
   </si>
   <si>
-    <t>Kombinovaná nejistota:</t>
-  </si>
-  <si>
     <t xml:space="preserve">                                                                           Nejistota typu B (měření probíhalo v obou případech posuvným měřítkem (odchylka 20μm):</t>
   </si>
   <si>
     <t>Nejpravděpodbnější objem(mm³):</t>
+  </si>
+  <si>
+    <t>Kombinovaná nejistota výsledného objemu:</t>
   </si>
 </sst>
 </file>
@@ -510,7 +510,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -524,6 +524,66 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -542,42 +602,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -585,59 +617,26 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -776,8 +775,8 @@
       <xdr:rowOff>111971</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="770659" cy="181460"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="TextBox 4">
@@ -819,6 +818,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -941,7 +941,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="TextBox 4">
@@ -1012,8 +1012,8 @@
       <xdr:rowOff>20822</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="897362" cy="316882"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="TextBox 5">
@@ -1055,6 +1055,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -1202,7 +1203,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="TextBox 5">
@@ -1285,7 +1286,7 @@
       <xdr:row>17</xdr:row>
       <xdr:rowOff>30444</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="1986378" cy="523348"/>
+    <xdr:ext cx="1914883" cy="523348"/>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
@@ -1302,7 +1303,7 @@
           <xdr:spPr>
             <a:xfrm>
               <a:off x="8192524" y="4709391"/>
-              <a:ext cx="1986378" cy="523348"/>
+              <a:ext cx="1914883" cy="523348"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -1484,7 +1485,21 @@
                         <m:nor/>
                       </m:rPr>
                       <a:rPr lang="en-US"/>
-                      <m:t>0,00577 </m:t>
+                      <m:t>0,005</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="cs-CZ" b="0" i="0"/>
+                      <m:t>8</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="en-US"/>
+                      <m:t> </m:t>
                     </m:r>
                     <m:r>
                       <m:rPr>
@@ -1552,7 +1567,7 @@
           <xdr:spPr>
             <a:xfrm>
               <a:off x="8192524" y="4709391"/>
-              <a:ext cx="1986378" cy="523348"/>
+              <a:ext cx="1914883" cy="523348"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -1633,7 +1648,19 @@
                 <a:rPr lang="en-US" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>0,00577 mm</a:t>
+                <a:t>0,005</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="cs-CZ" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>8</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> mm</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="en-US" i="0"/>
@@ -1682,8 +1709,8 @@
       <xdr:rowOff>52724</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2305888" cy="658514"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -1725,6 +1752,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2141,7 +2169,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="TextBox 7">
@@ -2205,8 +2233,8 @@
       <xdr:rowOff>156531</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3139449" cy="500137"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="TextBox 8">
@@ -2248,6 +2276,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -2713,7 +2742,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="TextBox 8">
@@ -2820,6 +2849,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -3156,6 +3186,7 @@
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -3166,7 +3197,7 @@
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                       </a:rPr>
-                      <m:t>≈7,70</m:t>
+                      <m:t>≈7,7</m:t>
                     </m:r>
                     <m:r>
                       <m:rPr>
@@ -3255,6 +3286,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -3266,11 +3298,12 @@
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>≈7,70" " 〖"mm" 〗^3</a:t>
+                <a:t>≈7,7" " 〖"mm" 〗^3</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -3331,6 +3364,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -3631,6 +3665,7 @@
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -3641,7 +3676,16 @@
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                       </a:rPr>
-                      <m:t>≈19,75</m:t>
+                      <m:t>≈</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>20</m:t>
                     </m:r>
                     <m:r>
                       <m:rPr>
@@ -3730,6 +3774,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -3741,11 +3786,24 @@
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>≈19,75" " 〖"mm" 〗^3</a:t>
+                <a:t>≈</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>"20</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> " 〖"mm" 〗^3</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -3806,6 +3864,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -4019,6 +4078,7 @@
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -4067,7 +4127,16 @@
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                       </a:rPr>
-                      <m:t>≈0,01665</m:t>
+                      <m:t>≈0,01</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>7</m:t>
                     </m:r>
                     <m:r>
                       <m:rPr>
@@ -4137,22 +4206,36 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>𝑢_𝐴 (¯𝑑)=√(1/(10⋅9) ∑24_(𝑖=1)^10▒(𝑑_𝑖−13,672)^2 )=</a:t>
+                <a:t>𝑢_𝐴 (¯𝑑)=√(1/(10⋅9) ∑_(𝑖=1)^10▒(𝑑_𝑖−13,672)^2 )=</a:t>
               </a:r>
               <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>√(0,02496/90)≈0,01665" mm"</a:t>
+                <a:t>√(0,02496/90)≈0,01</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>"7</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> mm"</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -4213,6 +4296,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -4426,6 +4510,7 @@
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -4474,7 +4559,7 @@
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                       </a:rPr>
-                      <m:t>≈0,00742</m:t>
+                      <m:t>≈0,0074</m:t>
                     </m:r>
                     <m:r>
                       <m:rPr>
@@ -4544,22 +4629,24 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>𝑢_𝐴 (¯ℎ)=√(1/(10⋅9) ∑24_(𝑖=1)^10▒(ℎ_𝑖−20,008)^2 )=</a:t>
+                <a:t>𝑢_𝐴 (¯ℎ)=√(1/(10⋅9) ∑_(𝑖=1)^10▒(ℎ_𝑖−20,008)^2 )=</a:t>
               </a:r>
               <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>√(0,00496/90)≈0,00742" mm"</a:t>
+                <a:t>√(0,00496/90)≈0,0074" mm"</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -4620,6 +4707,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -4833,6 +4921,7 @@
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -4881,7 +4970,16 @@
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                       </a:rPr>
-                      <m:t>≈0,01978</m:t>
+                      <m:t>≈0,0</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>20</m:t>
                     </m:r>
                     <m:r>
                       <m:rPr>
@@ -4951,22 +5049,36 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>𝑢_𝐴 (¯𝑎)=√(1/(10⋅9) ∑24_(𝑖=1)^10▒(𝑎_𝑖−11,700)^2 )=</a:t>
+                <a:t>𝑢_𝐴 (¯𝑎)=√(1/(10⋅9) ∑_(𝑖=1)^10▒(𝑎_𝑖−11,700)^2 )=</a:t>
               </a:r>
               <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>√(0,03520/90)≈0,01978" mm"</a:t>
+                <a:t>√(0,03520/90)≈0,0</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>"20</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> mm"</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -5027,6 +5139,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -5240,6 +5353,7 @@
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -5288,7 +5402,16 @@
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                       </a:rPr>
-                      <m:t>≈0,00846</m:t>
+                      <m:t>≈0,008</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>5</m:t>
                     </m:r>
                     <m:r>
                       <m:rPr>
@@ -5358,22 +5481,36 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>𝑢_𝐴 (¯𝑏)=√(1/(10⋅9) ∑24_(𝑖=1)^10▒(𝑏_𝑖−27,486)^2 )=</a:t>
+                <a:t>𝑢_𝐴 (¯𝑏)=√(1/(10⋅9) ∑_(𝑖=1)^10▒(𝑏_𝑖−27,486)^2 )=</a:t>
               </a:r>
               <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>√(0,00644/90)≈0,00846" mm"</a:t>
+                <a:t>√(0,00644/90)≈0,008</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>"5</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> mm"</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -5434,6 +5571,7 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -5647,6 +5785,7 @@
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a14:m>
                 <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
                   <m:oMathParaPr>
@@ -5695,7 +5834,16 @@
                       <a:rPr lang="en-US" sz="1100" i="1">
                         <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                       </a:rPr>
-                      <m:t>≈0,02256</m:t>
+                      <m:t>≈0,02</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t>3</m:t>
                     </m:r>
                     <m:r>
                       <m:rPr>
@@ -5765,22 +5913,36 @@
             </a:bodyPr>
             <a:lstStyle/>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>𝑢_𝐴 (¯𝑐)=√(1/(10⋅9) ∑24_(𝑖=1)^10▒(𝑐_𝑖−31,570)^2 )=</a:t>
+                <a:t>𝑢_𝐴 (¯𝑐)=√(1/(10⋅9) ∑_(𝑖=1)^10▒(𝑐_𝑖−31,570)^2 )=</a:t>
               </a:r>
               <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
               </a:endParaRPr>
             </a:p>
             <a:p>
+              <a:pPr/>
               <a:r>
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>√(0,04580/90)≈0,02256" mm"</a:t>
+                <a:t>√(0,04580/90)≈0,02</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>"3</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> mm"</a:t>
               </a:r>
               <a:endParaRPr lang="en-US" sz="1100"/>
             </a:p>
@@ -6110,7 +6272,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{468333C8-8064-D14E-96D6-F476956B8A12}">
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.33203125" customWidth="1"/>
@@ -6124,29 +6286,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="16"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="40"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="11" t="s">
+      <c r="B2" s="36"/>
+      <c r="C2" s="37"/>
+      <c r="D2" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-      <c r="G2" s="13"/>
+      <c r="E2" s="36"/>
+      <c r="F2" s="36"/>
+      <c r="G2" s="37"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -6172,25 +6334,25 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A4" s="19">
+      <c r="A4" s="13">
         <v>1</v>
       </c>
-      <c r="B4" s="17">
+      <c r="B4" s="11">
         <v>13.72</v>
       </c>
-      <c r="C4" s="20">
+      <c r="C4" s="14">
         <v>20</v>
       </c>
-      <c r="D4" s="19">
+      <c r="D4" s="13">
         <v>1</v>
       </c>
-      <c r="E4" s="17">
+      <c r="E4" s="11">
         <v>11.78</v>
       </c>
-      <c r="F4" s="21">
+      <c r="F4" s="15">
         <v>27.5</v>
       </c>
-      <c r="G4" s="20">
+      <c r="G4" s="14">
         <v>31.54</v>
       </c>
     </row>
@@ -6210,7 +6372,7 @@
       <c r="E5" s="3">
         <v>11.66</v>
       </c>
-      <c r="F5" s="22">
+      <c r="F5" s="16">
         <v>27.46</v>
       </c>
       <c r="G5" s="8">
@@ -6233,7 +6395,7 @@
       <c r="E6" s="3">
         <v>11.78</v>
       </c>
-      <c r="F6" s="22">
+      <c r="F6" s="16">
         <v>27.52</v>
       </c>
       <c r="G6" s="8">
@@ -6256,7 +6418,7 @@
       <c r="E7" s="3">
         <v>11.6</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="16">
         <v>27.5</v>
       </c>
       <c r="G7" s="8">
@@ -6279,7 +6441,7 @@
       <c r="E8" s="3">
         <v>11.7</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="16">
         <v>27.48</v>
       </c>
       <c r="G8" s="8">
@@ -6302,7 +6464,7 @@
       <c r="E9" s="3">
         <v>11.68</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="16">
         <v>27.44</v>
       </c>
       <c r="G9" s="8">
@@ -6325,7 +6487,7 @@
       <c r="E10" s="3">
         <v>11.64</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="16">
         <v>27.46</v>
       </c>
       <c r="G10" s="8">
@@ -6348,7 +6510,7 @@
       <c r="E11" s="3">
         <v>11.7</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="16">
         <v>27.48</v>
       </c>
       <c r="G11" s="8">
@@ -6371,7 +6533,7 @@
       <c r="E12" s="3">
         <v>11.68</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="16">
         <v>27.5</v>
       </c>
       <c r="G12" s="8">
@@ -6394,7 +6556,7 @@
       <c r="E13" s="4">
         <v>11.78</v>
       </c>
-      <c r="F13" s="18">
+      <c r="F13" s="12">
         <v>27.52</v>
       </c>
       <c r="G13" s="10">
@@ -6420,7 +6582,7 @@
         <f>AVERAGE(E4:E13)</f>
         <v>11.7</v>
       </c>
-      <c r="F14" s="18">
+      <c r="F14" s="12">
         <f>AVERAGE(F4:F13)</f>
         <v>27.486000000000001</v>
       </c>
@@ -6430,136 +6592,83 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="34" t="s">
+      <c r="A15" s="44" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="39"/>
-      <c r="C15" s="40"/>
-      <c r="D15" s="38" t="s">
+      <c r="B15" s="46"/>
+      <c r="C15" s="48"/>
+      <c r="D15" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="41"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="37"/>
+      <c r="E15" s="51"/>
+      <c r="F15" s="46"/>
+      <c r="G15" s="32"/>
     </row>
     <row r="16" spans="1:8" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="35"/>
-      <c r="B16" s="48"/>
+      <c r="A16" s="45"/>
+      <c r="B16" s="47"/>
       <c r="C16" s="49"/>
-      <c r="D16" s="50"/>
-      <c r="E16" s="51"/>
-      <c r="F16" s="48"/>
-      <c r="G16" s="26"/>
+      <c r="D16" s="43"/>
+      <c r="E16" s="52"/>
+      <c r="F16" s="47"/>
+      <c r="G16" s="50"/>
     </row>
-    <row r="17" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="29"/>
-      <c r="C17" s="52">
+    <row r="17" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="41"/>
+      <c r="C17" s="18">
         <f>0.25*PI()*POWER(B14,2)*C14</f>
         <v>2937.363266901928</v>
       </c>
-      <c r="D17" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="E17" s="53"/>
-      <c r="F17" s="12">
+      <c r="D17" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" s="20"/>
+      <c r="F17" s="36">
         <f>E14*F14*G14</f>
         <v>10152.476333999999</v>
       </c>
-      <c r="G17" s="13"/>
+      <c r="G17" s="37"/>
     </row>
-    <row r="18" spans="1:10" ht="36" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="B18" s="31"/>
-      <c r="C18" s="31"/>
-      <c r="D18" s="32"/>
-      <c r="E18" s="32"/>
-      <c r="F18" s="32"/>
-      <c r="G18" s="33"/>
+    <row r="18" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="24"/>
     </row>
-    <row r="19" spans="1:10" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="46" t="s">
-        <v>12</v>
-      </c>
-      <c r="B19" s="42"/>
-      <c r="C19" s="44"/>
-      <c r="D19" s="46" t="s">
-        <v>12</v>
-      </c>
-      <c r="E19" s="36"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="27"/>
-      <c r="I19" s="27"/>
-      <c r="J19" s="27"/>
+    <row r="19" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="27"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="31"/>
+      <c r="F19" s="31"/>
+      <c r="G19" s="32"/>
     </row>
-    <row r="20" spans="1:10" ht="61" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="47"/>
-      <c r="B20" s="43"/>
-      <c r="C20" s="45"/>
-      <c r="D20" s="47"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A21" s="27"/>
-      <c r="B21" s="27"/>
-      <c r="C21" s="27"/>
-      <c r="D21" s="27"/>
-      <c r="E21" s="27"/>
-      <c r="F21" s="27"/>
-      <c r="G21" s="27"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="27"/>
-    </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A22" s="27"/>
-      <c r="B22" s="27"/>
-      <c r="C22" s="27"/>
-      <c r="D22" s="27"/>
-      <c r="E22" s="27"/>
-      <c r="F22" s="27"/>
-      <c r="G22" s="27"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="27"/>
-    </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A23" s="27"/>
-      <c r="B23" s="27"/>
-      <c r="C23" s="27"/>
-      <c r="D23" s="27"/>
-      <c r="E23" s="27"/>
-      <c r="F23" s="27"/>
-      <c r="G23" s="27"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="27"/>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A24" s="27"/>
-      <c r="B24" s="27"/>
-      <c r="C24" s="27"/>
-      <c r="D24" s="27"/>
-      <c r="E24" s="27"/>
-      <c r="F24" s="27"/>
-      <c r="G24" s="27"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="27"/>
+    <row r="20" spans="1:9" ht="61" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="26"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="30"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="33"/>
+      <c r="F20" s="33"/>
+      <c r="G20" s="34"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:C20"/>
-    <mergeCell ref="E19:G20"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="D2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -6572,6 +6681,12 @@
     <mergeCell ref="F15:F16"/>
     <mergeCell ref="E15:E16"/>
     <mergeCell ref="F17:G17"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:C20"/>
+    <mergeCell ref="E19:G20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
vault backup: 2026-03-13 13:53:10
</commit_message>
<xml_diff>
--- a/FY1/1/FY1 - LAB1.xlsx
+++ b/FY1/1/FY1 - LAB1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marian/Documents/Zapisky/FY1/1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74CEBC7E-243B-1145-ABAC-24D070CB8BED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A9C4650-122C-9442-9D0A-26F8E5BA7634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{50D1F2D1-F177-9540-9CCC-CA14B3043CC0}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="16">
   <si>
     <t>Marian Frýba</t>
   </si>
@@ -82,6 +82,9 @@
   <si>
     <t>Kombinovaná nejistota výsledného objemu:</t>
   </si>
+  <si>
+    <t>Kombinovaná nejistota (mm):</t>
+  </si>
 </sst>
 </file>
 
@@ -109,7 +112,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="34">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -506,11 +509,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -546,12 +562,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
@@ -637,6 +647,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1705,7 +1727,7 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1135109</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>52724</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2305888" cy="658514"/>
@@ -2229,7 +2251,7 @@
     <xdr:from>
       <xdr:col>4</xdr:col>
       <xdr:colOff>1930633</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>19</xdr:row>
       <xdr:rowOff>156531</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3139449" cy="500137"/>
@@ -2802,10 +2824,10 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>212172</xdr:colOff>
-      <xdr:row>19</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>50191</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="4270592" cy="677301"/>
+    <xdr:ext cx="4114331" cy="677301"/>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
@@ -2821,8 +2843,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="1604716" y="5943437"/>
-              <a:ext cx="4270592" cy="677301"/>
+              <a:off x="1560154" y="6333349"/>
+              <a:ext cx="4114331" cy="677301"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3021,7 +3043,7 @@
                               <a:rPr lang="en-US" sz="1100" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>0,00940</m:t>
+                              <m:t>0,0094</m:t>
                             </m:r>
                           </m:e>
                           <m:sup>
@@ -3164,7 +3186,13 @@
                               <a:rPr lang="en-US" sz="1100" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>0,01763</m:t>
+                              <m:t>0,01</m:t>
+                            </m:r>
+                            <m:r>
+                              <a:rPr lang="cs-CZ" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>8</m:t>
                             </m:r>
                           </m:e>
                           <m:sup>
@@ -3258,8 +3286,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="1604716" y="5943437"/>
-              <a:ext cx="4270592" cy="677301"/>
+              <a:off x="1560154" y="6333349"/>
+              <a:ext cx="4114331" cy="677301"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3291,7 +3319,25 @@
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>𝑢_𝐶 (¯𝑉)=√((𝜋^2⋅〖13,672〗^4)/16⋅〖0,00940〗^2+(𝜋^2⋅〖13,672〗^2⋅〖20,008〗^2)/4⋅〖0,01763〗^2 )</a:t>
+                <a:t>𝑢_𝐶 (¯𝑉)=√((𝜋^2⋅〖13,672〗^4)/16⋅〖0,0094〗^2+(𝜋^2⋅〖13,672〗^2⋅〖20,008〗^2)/4⋅〖0,01</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>8</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>〗^</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>2 )</a:t>
               </a:r>
               <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
@@ -3316,11 +3362,11 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>278824</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>166662</xdr:rowOff>
+      <xdr:colOff>668736</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>55259</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="6396944" cy="392415"/>
+    <xdr:ext cx="5423280" cy="557781"/>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
       <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
@@ -3336,8 +3382,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="7397508" y="6059908"/>
-              <a:ext cx="6396944" cy="392415"/>
+              <a:off x="7742859" y="6338417"/>
+              <a:ext cx="5423280" cy="557781"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3464,7 +3510,7 @@
                                   <a:rPr lang="en-US" sz="1100" i="1">
                                     <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                   </a:rPr>
-                                  <m:t>27,486⋅31,570</m:t>
+                                  <m:t>27,486⋅31,57</m:t>
                                 </m:r>
                               </m:e>
                             </m:d>
@@ -3497,7 +3543,13 @@
                               <a:rPr lang="en-US" sz="1100" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>0,02060</m:t>
+                              <m:t>0,02</m:t>
+                            </m:r>
+                            <m:r>
+                              <a:rPr lang="cs-CZ" sz="1100" b="0" i="1">
+                                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                              </a:rPr>
+                              <m:t>1</m:t>
                             </m:r>
                           </m:e>
                           <m:sup>
@@ -3537,7 +3589,7 @@
                                   <a:rPr lang="en-US" sz="1100" i="1">
                                     <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                   </a:rPr>
-                                  <m:t>11,700⋅31,570</m:t>
+                                  <m:t>11,7⋅31,57</m:t>
                                 </m:r>
                               </m:e>
                             </m:d>
@@ -3570,7 +3622,7 @@
                               <a:rPr lang="en-US" sz="1100" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>0,01024</m:t>
+                              <m:t>0,01</m:t>
                             </m:r>
                           </m:e>
                           <m:sup>
@@ -3610,7 +3662,7 @@
                                   <a:rPr lang="en-US" sz="1100" i="1">
                                     <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                                   </a:rPr>
-                                  <m:t>11,700⋅27,486</m:t>
+                                  <m:t>11,7⋅27,486</m:t>
                                 </m:r>
                               </m:e>
                             </m:d>
@@ -3643,7 +3695,7 @@
                               <a:rPr lang="en-US" sz="1100" i="1">
                                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               </a:rPr>
-                              <m:t>0,02329</m:t>
+                              <m:t>0,023</m:t>
                             </m:r>
                           </m:e>
                           <m:sup>
@@ -3660,6 +3712,12 @@
                   </m:oMath>
                 </m:oMathPara>
               </a14:m>
+              <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:pPr/>
               <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
               </a:endParaRPr>
@@ -3746,8 +3804,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="7397508" y="6059908"/>
-              <a:ext cx="6396944" cy="392415"/>
+              <a:off x="7742859" y="6338417"/>
+              <a:ext cx="5423280" cy="557781"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -3779,8 +3837,32 @@
                 <a:rPr lang="en-US" sz="1100" i="0">
                   <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                 </a:rPr>
-                <a:t>𝑢_𝐶 (¯𝑉)=√((27,486⋅31,570)^2⋅〖0,02060〗^2+(11,700⋅31,570)^2⋅〖0,01024〗^2+(11,700⋅27,486)^2⋅〖0,02329〗^2 )</a:t>
+                <a:t>𝑢_𝐶 (¯𝑉)=√((27,486⋅31,57)^2⋅〖0,02</a:t>
               </a:r>
+              <a:r>
+                <a:rPr lang="cs-CZ" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>1</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>〗^</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="en-US" sz="1100" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t>2+(11,7⋅31,57)^2⋅〖0,01〗^2+(11,7⋅27,486)^2⋅〖0,023〗^2 )</a:t>
+              </a:r>
+              <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
+                <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+            <a:p>
+              <a:pPr/>
               <a:endParaRPr lang="cs-CZ" sz="1100" i="1">
                 <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
               </a:endParaRPr>
@@ -6272,10 +6354,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{468333C8-8064-D14E-96D6-F476956B8A12}">
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="13.33203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" customWidth="1"/>
     <col min="2" max="2" width="30.1640625" customWidth="1"/>
     <col min="3" max="3" width="30.6640625" customWidth="1"/>
     <col min="4" max="4" width="14.33203125" customWidth="1"/>
@@ -6286,29 +6368,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="32" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="40"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="38"/>
       <c r="H1" s="1"/>
     </row>
     <row r="2" spans="1:8" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="33" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="36"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="35" t="s">
+      <c r="B2" s="34"/>
+      <c r="C2" s="35"/>
+      <c r="D2" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="37"/>
+      <c r="E2" s="34"/>
+      <c r="F2" s="34"/>
+      <c r="G2" s="35"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="5" t="s">
@@ -6592,32 +6674,32 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="44" t="s">
+      <c r="A15" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="46"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="42" t="s">
+      <c r="B15" s="44"/>
+      <c r="C15" s="46"/>
+      <c r="D15" s="40" t="s">
         <v>11</v>
       </c>
-      <c r="E15" s="51"/>
-      <c r="F15" s="46"/>
-      <c r="G15" s="32"/>
+      <c r="E15" s="49"/>
+      <c r="F15" s="44"/>
+      <c r="G15" s="30"/>
     </row>
     <row r="16" spans="1:8" ht="39" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="45"/>
-      <c r="B16" s="47"/>
-      <c r="C16" s="49"/>
-      <c r="D16" s="43"/>
-      <c r="E16" s="52"/>
-      <c r="F16" s="47"/>
-      <c r="G16" s="50"/>
+      <c r="A16" s="43"/>
+      <c r="B16" s="45"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="41"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="45"/>
+      <c r="G16" s="48"/>
     </row>
     <row r="17" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="B17" s="41"/>
+      <c r="B17" s="39"/>
       <c r="C17" s="18">
         <f>0.25*PI()*POWER(B14,2)*C14</f>
         <v>2937.363266901928</v>
@@ -6626,11 +6708,11 @@
         <v>13</v>
       </c>
       <c r="E17" s="20"/>
-      <c r="F17" s="36">
+      <c r="F17" s="34">
         <f>E14*F14*G14</f>
         <v>10152.476333999999</v>
       </c>
-      <c r="G17" s="37"/>
+      <c r="G17" s="35"/>
     </row>
     <row r="18" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="21" t="s">
@@ -6638,34 +6720,57 @@
       </c>
       <c r="B18" s="22"/>
       <c r="C18" s="22"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="24"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="52"/>
     </row>
-    <row r="19" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="25" t="s">
+    <row r="19" spans="1:9" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="51" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="53">
+        <v>1.7999999999999999E-2</v>
+      </c>
+      <c r="C19" s="54">
+        <v>9.4000000000000004E-3</v>
+      </c>
+      <c r="D19" s="51" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" s="53">
+        <v>2.1000000000000001E-2</v>
+      </c>
+      <c r="F19" s="53">
+        <v>0.01</v>
+      </c>
+      <c r="G19" s="54">
+        <v>2.3E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="60" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="27"/>
-      <c r="C19" s="28"/>
-      <c r="D19" s="25" t="s">
+      <c r="B20" s="25"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="31"/>
-      <c r="F19" s="31"/>
-      <c r="G19" s="32"/>
+      <c r="E20" s="29"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="30"/>
     </row>
-    <row r="20" spans="1:9" ht="61" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="26"/>
-      <c r="B20" s="29"/>
-      <c r="C20" s="30"/>
-      <c r="D20" s="26"/>
-      <c r="E20" s="33"/>
-      <c r="F20" s="33"/>
-      <c r="G20" s="34"/>
-      <c r="H20" s="17"/>
-      <c r="I20" s="17"/>
+    <row r="21" spans="1:9" ht="61" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="24"/>
+      <c r="B21" s="27"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="24"/>
+      <c r="E21" s="31"/>
+      <c r="F21" s="31"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="17"/>
+      <c r="I21" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="18">
@@ -6683,10 +6788,10 @@
     <mergeCell ref="F17:G17"/>
     <mergeCell ref="D17:E17"/>
     <mergeCell ref="A18:G18"/>
-    <mergeCell ref="D19:D20"/>
-    <mergeCell ref="A19:A20"/>
-    <mergeCell ref="B19:C20"/>
-    <mergeCell ref="E19:G20"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:C21"/>
+    <mergeCell ref="E20:G21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>